<commit_message>
Add dashboard attention section
</commit_message>
<xml_diff>
--- a/generated/powerbi_movimentacoes.xlsx
+++ b/generated/powerbi_movimentacoes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK5"/>
+  <dimension ref="A1:AK6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1160,7 +1160,6 @@
           <t>AT/PM</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>PCA</t>
@@ -1272,7 +1271,179 @@
           <t>ALMOXARIFADO-PRÉDIO 3-ADELAIDE</t>
         </is>
       </c>
-      <c r="AK5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-27 09:45:43</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SOLICITACAO</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GUILHERME BRAGA BRANGIONI</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Solicitação de empréstimo criada.</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>EMP-ATPM-20260527-0008</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PENDENTE_APROVACAO</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>GUILHERME BRAGA BRANGIONI</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>59748</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>guilherme.bbrangioni@cemig.com.br</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>31998838780</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>AT/PM</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>PCA</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>GUILHERME BRAGA BRANGIONI</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>guilherme.bbrangioni@cemig.com.br</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>GUILHERME BRAGA BRANGIONI</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>guilherme.bbrangioni@cemig.com.br</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>2026-05-27 12:45:20</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>2026-05-29 00:00:00</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>LABORATORIO AT/PM</t>
+        </is>
+      </c>
+      <c r="W6" t="n">
+        <v>8</v>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>EMPRESTADO</t>
+        </is>
+      </c>
+      <c r="Y6" t="n">
+        <v>155</v>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>EQP-0155</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>RELÉ DE PROTEÇÃO DE LINHA</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>7SA87</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>P1A433914</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>BM2507001259</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>RESERVADO</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>AT/PM</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>ALMOXARIFADO-PRÉDIO 3-ADELAIDE</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>BARREIRO</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add filters in users page
</commit_message>
<xml_diff>
--- a/generated/powerbi_movimentacoes.xlsx
+++ b/generated/powerbi_movimentacoes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK6"/>
+  <dimension ref="A1:AK8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1331,7 +1331,6 @@
           <t>AT/PM</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>PCA</t>
@@ -1367,7 +1366,6 @@
           <t>2026-05-29 00:00:00</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
           <t>LABORATORIO AT/PM</t>
@@ -1440,6 +1438,340 @@
         </is>
       </c>
       <c r="AK6" t="inlineStr">
+        <is>
+          <t>BARREIRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-27 15:34:08</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DEVOLUCAO_TOTAL</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>André José Soares Costa</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Devolução total registrada.</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>EMP-20260525-0006</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>FINALIZADO</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ANDRÉ JOSÉ SOARES COSTA</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>59723</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>andre.jcosta@cemig.com.br</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>EI/PO</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>COMISSIONAMENTO</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>GUILHERME BRAGA BRANGIONI</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>guilherme.bbrangioni@cemig.com.br</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>GUILHERME BRAGA BRANGIONI</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>2026-05-25 16:32:21</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>2026-05-27 18:28:28</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>LABORATÓRIO COMISSIONAMENTO</t>
+        </is>
+      </c>
+      <c r="W7" t="n">
+        <v>6</v>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>DEVOLVIDO</t>
+        </is>
+      </c>
+      <c r="Y7" t="n">
+        <v>158</v>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>EQP-0158</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>MÓDULO DE AQUISIÇÃO</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>GE</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>RA332</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>RA3323666622CC</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>DISPONIVEL</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>ALMOXARIFADO-PRÉDIO 3-ADELAIDE</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>ITAJUBÁ 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-27 15:34:09</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>REJEICAO</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Guilherme Braga Brangioni</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Equipamento em uso</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>8</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>EMP-ATPM-20260527-0008</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>REJEITADO</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>GUILHERME BRAGA BRANGIONI</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>59748</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>guilherme.bbrangioni@cemig.com.br</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>31998838780</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>AT/PM</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>PCA</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>GUILHERME BRAGA BRANGIONI</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>guilherme.bbrangioni@cemig.com.br</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>GUILHERME BRAGA BRANGIONI</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>guilherme.bbrangioni@cemig.com.br</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>2026-05-27 12:45:20</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>2026-05-29 00:00:00</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>LABORATORIO AT/PM</t>
+        </is>
+      </c>
+      <c r="W8" t="n">
+        <v>8</v>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>CANCELADO</t>
+        </is>
+      </c>
+      <c r="Y8" t="n">
+        <v>155</v>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>EQP-0155</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>RELÉ DE PROTEÇÃO DE LINHA</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>7SA87</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>P1A433914</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>BM2507001259</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>DISPONIVEL</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>AT/PM</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>ALMOXARIFADO-PRÉDIO 3-ADELAIDE</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
         <is>
           <t>BARREIRO</t>
         </is>

</xml_diff>

<commit_message>
Revert network deployment and keep local execution
</commit_message>
<xml_diff>
--- a/generated/powerbi_movimentacoes.xlsx
+++ b/generated/powerbi_movimentacoes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK8"/>
+  <dimension ref="A1:AK11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1663,7 +1663,6 @@
           <t>AT/PM</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
           <t>PCA</t>
@@ -1699,7 +1698,6 @@
           <t>2026-05-29 00:00:00</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
           <t>LABORATORIO AT/PM</t>
@@ -1776,6 +1774,451 @@
           <t>BARREIRO</t>
         </is>
       </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-05-28 09:57:42</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SOLICITACAO</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ÁLVARO RODRIGO GUIMARÃES SILVA</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Solicitação de empréstimo criada.</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>9</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>EMP-ATPM-20260528-0009</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>RETIRADO</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>ALVARO RODRIGO</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>60492</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>alvaro.rsilva@cemig.com.br</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>GUILHERME BRAGA BRANGIONI</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>guilherme.bbrangioni@cemig.com.br</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>ÁLVARO RODRIGO GUIMARÃES SILVA</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>alvaro.rsilva@cemig.com.br</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:42:46</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>2026-05-30 00:00:00</t>
+        </is>
+      </c>
+      <c r="W9" t="n">
+        <v>9</v>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>EMPRESTADO</t>
+        </is>
+      </c>
+      <c r="Y9" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>EQP-0007</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>RELÉ DE PROTEÇÃO DE TRANSFORMADOR</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>NARI</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>PCS-978</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>PCS-978-I-EN-5A-170708</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>NRJB2135751920040</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>EMPRESTADO</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>AT/PM</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>ALMOXARIFADO-PRÉDIO 3-ADELAIDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-28 09:57:42</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>APROVACAO</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Guilherme Braga Brangioni</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Solicitação aprovada pelo sistema.</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>9</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>EMP-ATPM-20260528-0009</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>RETIRADO</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ALVARO RODRIGO</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>60492</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>alvaro.rsilva@cemig.com.br</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>GUILHERME BRAGA BRANGIONI</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>guilherme.bbrangioni@cemig.com.br</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>ÁLVARO RODRIGO GUIMARÃES SILVA</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>alvaro.rsilva@cemig.com.br</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:42:46</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>2026-05-30 00:00:00</t>
+        </is>
+      </c>
+      <c r="W10" t="n">
+        <v>9</v>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>EMPRESTADO</t>
+        </is>
+      </c>
+      <c r="Y10" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>EQP-0007</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>RELÉ DE PROTEÇÃO DE TRANSFORMADOR</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>NARI</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>PCS-978</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>PCS-978-I-EN-5A-170708</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>NRJB2135751920040</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>EMPRESTADO</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>AT/PM</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>ALMOXARIFADO-PRÉDIO 3-ADELAIDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-05-28 09:57:43</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>RETIRADA</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Álvaro Rodrigo</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Retirada/coleta confirmada.</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>9</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>EMP-ATPM-20260528-0009</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>RETIRADO</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>ALVARO RODRIGO</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>60492</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>alvaro.rsilva@cemig.com.br</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>GUILHERME BRAGA BRANGIONI</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>guilherme.bbrangioni@cemig.com.br</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>ÁLVARO RODRIGO GUIMARÃES SILVA</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>alvaro.rsilva@cemig.com.br</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:42:46</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>2026-05-30 00:00:00</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="n">
+        <v>9</v>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>EMPRESTADO</t>
+        </is>
+      </c>
+      <c r="Y11" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>EQP-0007</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>RELÉ DE PROTEÇÃO DE TRANSFORMADOR</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>NARI</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>PCS-978</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>PCS-978-I-EN-5A-170708</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>NRJB2135751920040</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>EMPRESTADO</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>AT/PM</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>ALMOXARIFADO-PRÉDIO 3-ADELAIDE</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>